<commit_message>
auto: daily pipeline 2026-09-05 - 109 leads, 68 sent
</commit_message>
<xml_diff>
--- a/indian_hotel_leads.xlsx
+++ b/indian_hotel_leads.xlsx
@@ -711,7 +711,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Not listed on Maps</t>
+          <t>7009311130</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -2219,12 +2219,12 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Not listed on Maps</t>
+          <t>8743000181</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>booking@rchronline.com</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>sunsetbeachresortgoa@gmail.com</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>dunes13@rediffmail.com</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">

</xml_diff>

<commit_message>
auto: daily pipeline 2026-09-10 - 126 leads, 181 sent
</commit_message>
<xml_diff>
--- a/indian_hotel_leads.xlsx
+++ b/indian_hotel_leads.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J109"/>
+  <dimension ref="A1:J126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -575,7 +575,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -627,7 +627,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>support@scantrip.com</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>info@prospectpt.com</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>info@cliffecottage.com</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>info@paramounthotels.com</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>hari@gmail.com</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>contact@hotelgreenparkgoa.com</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
@@ -2447,7 +2447,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>contact@gtdchotel.com</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>hm@advanihotels.com</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
@@ -2811,7 +2811,7 @@
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
@@ -2863,7 +2863,7 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
@@ -2967,7 +2967,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -3019,7 +3019,7 @@
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I51" s="4" t="inlineStr">
@@ -3175,7 +3175,7 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I53" s="4" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -3435,7 +3435,7 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I57" s="4" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>reservations@sunnsandpune.com</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
@@ -3591,7 +3591,7 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>contact@sironamedical.com</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
@@ -3695,7 +3695,7 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I63" s="4" t="inlineStr">
@@ -3784,7 +3784,7 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>hotelraviraj@gmail.com</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
@@ -3799,7 +3799,7 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
@@ -3851,7 +3851,7 @@
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I65" s="4" t="inlineStr">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -3940,7 +3940,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>admissions.mitid@mituniversity.edu.in</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
@@ -3955,7 +3955,7 @@
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -4111,7 +4111,7 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
@@ -4148,7 +4148,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>admissions@iiserpune.ac.in</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I71" s="4" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>enquiry@vidyaniketanhostels.com</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
@@ -4215,7 +4215,7 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
@@ -4423,7 +4423,7 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -4460,7 +4460,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>meghmalhartourism@gmail.com</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
@@ -4475,7 +4475,7 @@
       </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
@@ -4527,7 +4527,7 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="H79" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
@@ -4772,7 +4772,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>chandrakantpatil0796@gmail.com</t>
         </is>
       </c>
       <c r="F83" s="5" t="inlineStr">
@@ -4787,7 +4787,7 @@
       </c>
       <c r="H83" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I83" s="4" t="inlineStr">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
@@ -4980,7 +4980,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>info@pankajdevelopers.com</t>
         </is>
       </c>
       <c r="F87" s="5" t="inlineStr">
@@ -4995,7 +4995,7 @@
       </c>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I87" s="4" t="inlineStr">
@@ -5032,7 +5032,7 @@
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>sales@jfe-eng.co.in</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
@@ -5047,7 +5047,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="H89" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I89" s="4" t="inlineStr">
@@ -5203,7 +5203,7 @@
       </c>
       <c r="H91" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I91" s="4" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>contactus@commonfloor.com</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
@@ -5255,7 +5255,7 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
@@ -5292,7 +5292,7 @@
       </c>
       <c r="E93" s="5" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>agency2050@gmail.com</t>
         </is>
       </c>
       <c r="F93" s="5" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="H93" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I93" s="4" t="inlineStr">
@@ -5344,7 +5344,7 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>contactus@commonfloor.com</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
@@ -5359,7 +5359,7 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
@@ -5411,7 +5411,7 @@
       </c>
       <c r="H95" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
@@ -5463,7 +5463,7 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr">
@@ -5515,7 +5515,7 @@
       </c>
       <c r="H97" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I97" s="4" t="inlineStr">
@@ -5552,7 +5552,7 @@
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>contactus@commonfloor.com</t>
         </is>
       </c>
       <c r="F98" s="3" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
@@ -5656,7 +5656,7 @@
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>support@beyondwalls.com</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
@@ -5671,7 +5671,7 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="H101" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I101" s="4" t="inlineStr">
@@ -6020,7 +6020,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>mhrs.pnqms.reservation@marriotthotels.com</t>
         </is>
       </c>
       <c r="F107" s="5" t="inlineStr">
@@ -6035,7 +6035,7 @@
       </c>
       <c r="H107" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I107" s="4" t="inlineStr">
@@ -6072,7 +6072,7 @@
       </c>
       <c r="E108" s="3" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>a@diat.ac.in</t>
         </is>
       </c>
       <c r="F108" s="3" t="inlineStr">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr">
@@ -6124,7 +6124,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t>Pending lookup</t>
+          <t>info@cloudninecare.com</t>
         </is>
       </c>
       <c r="F109" s="5" t="inlineStr">
@@ -6139,7 +6139,7 @@
       </c>
       <c r="H109" s="4" t="inlineStr">
         <is>
-          <t>IDENTIFIED</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="I109" s="4" t="inlineStr">
@@ -6150,6 +6150,890 @@
       <c r="J109" s="5" t="inlineStr">
         <is>
           <t>Indian Camp Site in Pune. No standalone booking website. High MakeMyTrip/OTA commission loss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>us-serper-0109</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>Contact us</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>Not listed on Maps</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>info@hotelboutiqueny.com</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hotelboutiqueatgrandcentral.com/contact/</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J110" s="3" t="inlineStr">
+        <is>
+          <t>USA independent hotel in New York found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>us-serper-0110</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>Not listed on Maps</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>reservations@hotelatfifthavenyc.com</t>
+        </is>
+      </c>
+      <c r="F111" s="5" t="inlineStr">
+        <is>
+          <t>https://www.hotelatfifthavenuenyc.com/contact</t>
+        </is>
+      </c>
+      <c r="G111" s="4" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H111" s="4" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I111" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J111" s="5" t="inlineStr">
+        <is>
+          <t>USA independent hotel in New York found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>us-serper-0111</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>Contact Information</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>Not listed on Maps</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>FiftyFD@sonesta.com</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>NO WEBSITE (OTA Only)</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J112" s="3" t="inlineStr">
+        <is>
+          <t>USA independent hotel in New York found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>us-serper-0112</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>Contact The Mark Hotel NYC</t>
+        </is>
+      </c>
+      <c r="C113" s="4" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>+1 866 744 4300</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>FiftyFD@sonesta.com</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>https://www.themarkhotel.com/information/contact/</t>
+        </is>
+      </c>
+      <c r="G113" s="4" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H113" s="4" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I113" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J113" s="5" t="inlineStr">
+        <is>
+          <t>USA independent hotel in New York found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>us-serper-0113</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>Does anyone have an email address for Ne</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>Not listed on Maps</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>reservations@themarkhotel.com</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>NO WEBSITE (OTA Only)</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J114" s="3" t="inlineStr">
+        <is>
+          <t>USA independent hotel in New York found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>us-serper-0114</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>Crowne Plaza Manhattan Times Square</t>
+        </is>
+      </c>
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>+1-212-5813300</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>nynyreservations@nynyvegas.com</t>
+        </is>
+      </c>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ihg.com/crowneplaza/hotels/us/en/new-york/nycat/hoteldetail</t>
+        </is>
+      </c>
+      <c r="G115" s="4" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H115" s="4" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I115" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J115" s="5" t="inlineStr">
+        <is>
+          <t>USA independent hotel in New York found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>us-serper-0115</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>Arthouse Hotel</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>+1 212-362-1100</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>reservations@cptsnyc.com</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>https://www.arthousehotelnyc.com/</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J116" s="3" t="inlineStr">
+        <is>
+          <t>USA independent hotel in New York found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>us-serper-0116</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>Hotels in New York City</t>
+        </is>
+      </c>
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>Not listed on Maps</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>connect@arthousehotelnyc.com</t>
+        </is>
+      </c>
+      <c r="F117" s="5" t="inlineStr">
+        <is>
+          <t>https://www.themusehotel.com/contact-us</t>
+        </is>
+      </c>
+      <c r="G117" s="4" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H117" s="4" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I117" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J117" s="5" t="inlineStr">
+        <is>
+          <t>USA independent hotel in New York found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>us-serper-0117</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>Public Hotel New York</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>Not listed on Maps</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>talktous@themusehotel.com</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr">
+        <is>
+          <t>https://www.publichotels.com/newyork/contact</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J118" s="3" t="inlineStr">
+        <is>
+          <t>USA independent hotel in New York found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>us-serper-0118</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>Luxury Miami Hotels</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>Not listed on Maps</t>
+        </is>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>reservationsny@publichotels.com</t>
+        </is>
+      </c>
+      <c r="F119" s="5" t="inlineStr">
+        <is>
+          <t>https://www.icmiamihotel.com/contact</t>
+        </is>
+      </c>
+      <c r="G119" s="4" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H119" s="4" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I119" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J119" s="5" t="inlineStr">
+        <is>
+          <t>USA independent hotel in Miami found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>us-serper-0119</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>The Miami Beach EDITION</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>+1 786 257 4500</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>MiamiBilling@ihg.com</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>https://www.editionhotels.com/miami-beach/</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J120" s="3" t="inlineStr">
+        <is>
+          <t>USA independent hotel in Miami found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>us-serper-0120</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>the goodtime hotel, Miami Beach, a Tribu</t>
+        </is>
+      </c>
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>+1 786-687-0234</t>
+        </is>
+      </c>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>hotelnewyorkermiami@gmail.com</t>
+        </is>
+      </c>
+      <c r="F121" s="5" t="inlineStr">
+        <is>
+          <t>https://www.marriott.com/en-us/hotels/miasx-the-goodtime-hotel-miami-beach-a-tribute-portfolio-hotel/overview/</t>
+        </is>
+      </c>
+      <c r="G121" s="4" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H121" s="4" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I121" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J121" s="5" t="inlineStr">
+        <is>
+          <t>USA independent hotel in Miami found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>us-serper-0121</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>Contact Us</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>+1(786)913 0680</t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>info@esmehotel.com</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="inlineStr">
+        <is>
+          <t>NO WEBSITE (OTA Only)</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J122" s="3" t="inlineStr">
+        <is>
+          <t>USA independent hotel in Miami found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>us-serper-0122</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>Luxury Boutique Hotel Close to South Bea</t>
+        </is>
+      </c>
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>Not listed on Maps</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>frontdesk@hoteltrouvail.com</t>
+        </is>
+      </c>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>https://www.esmehotel.com/</t>
+        </is>
+      </c>
+      <c r="G123" s="4" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H123" s="4" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I123" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J123" s="5" t="inlineStr">
+        <is>
+          <t>USA independent hotel in Miami found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>us-serper-0123</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>Contact Us Today</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>Not listed on Maps</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>frontdesk@hoteltrouvail.com</t>
+        </is>
+      </c>
+      <c r="F124" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hoteltrouvailmiamibeach.com/get-in-touch</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J124" s="3" t="inlineStr">
+        <is>
+          <t>USA independent hotel in Miami found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="inlineStr">
+        <is>
+          <t>us-serper-0124</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>Contact Us</t>
+        </is>
+      </c>
+      <c r="C125" s="4" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D125" s="4" t="inlineStr">
+        <is>
+          <t>Not listed on Maps</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>stay@slh.com</t>
+        </is>
+      </c>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>NO WEBSITE (OTA Only)</t>
+        </is>
+      </c>
+      <c r="G125" s="4" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H125" s="4" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I125" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J125" s="5" t="inlineStr">
+        <is>
+          <t>USA independent hotel in Los Angeles found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>us-serper-0125</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>Contact Us</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>Las Vegas</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>Not listed on Maps</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>frontdesk@serenevegas.com</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>NO WEBSITE (OTA Only)</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>18% - 22% (MakeMyTrip/Goibibo)</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="J126" s="3" t="inlineStr">
+        <is>
+          <t>USA independent hotel in Las Vegas found via live Google Search. No direct booking site. Losing 15-25% to Booking.com/Expedia.</t>
         </is>
       </c>
     </row>

</xml_diff>